<commit_message>
discu + intro parties + embed
</commit_message>
<xml_diff>
--- a/Figures/Bad_Chinchilloids_from_Carrillo.xlsx
+++ b/Figures/Bad_Chinchilloids_from_Carrillo.xlsx
@@ -34,60 +34,38 @@
     <t xml:space="preserve">Cephalomyopsis_hipselodontus</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Typo (h</t>
-    </r>
+    <t xml:space="preserve">Typo (h**y**pselodontus, not h**i**pselodontus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discolomys_cuneus</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
-        <u val="single"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">y</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">pselodontus, not hipselodontus)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Discolomys_cuneus</t>
-  </si>
-  <si>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Discolomys cuneus</t>
+    </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">“</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Discolomys cuneus</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">”</t>
     </r>
@@ -96,6 +74,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> (missing open nomenclature)</t>
     </r>
@@ -115,6 +94,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Forgotten “?” → </t>
     </r>
@@ -124,6 +104,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">?G. quadratus</t>
     </r>
@@ -137,6 +118,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Forgotten “?” → </t>
     </r>
@@ -146,6 +128,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">?G. royoi</t>
     </r>
@@ -159,6 +142,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Synonym of </t>
     </r>
@@ -168,6 +152,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Drytomomys</t>
     </r>
@@ -179,32 +164,7 @@
     <t xml:space="preserve">Scleromys_osbornianus</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Typo (osbornia</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <u val="single"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">t</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">us, not osbornianus)</t>
-    </r>
+    <t xml:space="preserve">Typo (osbornia**t**us, not osbornia**n**us)</t>
   </si>
   <si>
     <t xml:space="preserve">Sphigomys_zonatus</t>
@@ -230,6 +190,7 @@
         <sz val="10"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Tetrastylopsis araucanus according to</t>
     </r>
@@ -239,6 +200,7 @@
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> Arnal &amp; Pérez (2025) − but see Nasif, (2009); Sostillo et al., (2022): Tetrastylus araucanus</t>
     </r>
@@ -263,11 +225,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -289,25 +252,21 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <u val="single"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -358,20 +317,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -573,110 +536,110 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="2" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>